<commit_message>
simulation to initialize Wheat-BRIDGES
</commit_message>
<xml_diff>
--- a/simulations/scene/inputs/Scenarios_25_08_08.xlsx
+++ b/simulations/scene/inputs/Scenarios_25_08_08.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp29072\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\scene\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TIGERA~1\AppData\Local\Temp\scp10384\home\torisuten\package\Wheat-BRIDGES\Root_BRIDGES\simulations\scene\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23095EF4-EEB8-4B51-8070-1C5FF664E537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C6178B-F119-4188-9F90-A9F2DCBE0AC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3427,7 +3427,7 @@
         <v>604</v>
       </c>
       <c r="M8" s="36">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="N8" s="36">
         <v>0</v>
@@ -14862,7 +14862,7 @@
       </c>
       <c r="K226" s="83"/>
       <c r="L226" s="83">
-        <f t="shared" ref="L226:M226" si="24">0.00001</f>
+        <f t="shared" ref="L226" si="24">0.00001</f>
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="M226" s="83">
@@ -15417,7 +15417,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G236:I237">
-    <cfRule type="colorScale" priority="23">
+    <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15427,7 +15427,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="24">
+    <cfRule type="colorScale" priority="23">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15439,7 +15439,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G237:N237">
-    <cfRule type="colorScale" priority="552">
+    <cfRule type="colorScale" priority="553">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15449,7 +15449,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="553">
+    <cfRule type="colorScale" priority="552">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15473,7 +15473,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H213:N213">
-    <cfRule type="colorScale" priority="558">
+    <cfRule type="colorScale" priority="559">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15483,7 +15483,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="559">
+    <cfRule type="colorScale" priority="558">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15495,7 +15495,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H214:N214">
-    <cfRule type="colorScale" priority="562">
+    <cfRule type="colorScale" priority="563">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15505,7 +15505,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="563">
+    <cfRule type="colorScale" priority="562">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15539,7 +15539,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H216:N216">
-    <cfRule type="colorScale" priority="570">
+    <cfRule type="colorScale" priority="571">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15549,7 +15549,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="571">
+    <cfRule type="colorScale" priority="570">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15561,7 +15561,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H217:N217">
-    <cfRule type="colorScale" priority="574">
+    <cfRule type="colorScale" priority="575">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15571,7 +15571,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="575">
+    <cfRule type="colorScale" priority="574">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15583,7 +15583,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H218:N218">
-    <cfRule type="colorScale" priority="578">
+    <cfRule type="colorScale" priority="579">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15593,7 +15593,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="579">
+    <cfRule type="colorScale" priority="578">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15605,7 +15605,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H221:N221">
-    <cfRule type="colorScale" priority="582">
+    <cfRule type="colorScale" priority="583">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15615,7 +15615,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="583">
+    <cfRule type="colorScale" priority="582">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15627,7 +15627,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H223:N224 H222:L222 N222">
-    <cfRule type="colorScale" priority="586">
+    <cfRule type="colorScale" priority="587">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15637,7 +15637,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="587">
+    <cfRule type="colorScale" priority="586">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15649,7 +15649,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H225:N225">
-    <cfRule type="colorScale" priority="590">
+    <cfRule type="colorScale" priority="591">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15659,7 +15659,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="591">
+    <cfRule type="colorScale" priority="590">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15737,7 +15737,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K228:M228">
-    <cfRule type="colorScale" priority="602">
+    <cfRule type="colorScale" priority="603">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15747,7 +15747,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="603">
+    <cfRule type="colorScale" priority="602">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15759,6 +15759,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K236:N237">
+    <cfRule type="colorScale" priority="605">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="604">
       <colorScale>
         <cfvo type="min"/>
@@ -15769,7 +15779,41 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="605">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M222">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M226">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15815,7 +15859,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q132:R132 H132:O132">
-    <cfRule type="colorScale" priority="303">
+    <cfRule type="colorScale" priority="304">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15825,7 +15869,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="304">
+    <cfRule type="colorScale" priority="303">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15837,7 +15881,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q133:R133 H133:N133">
-    <cfRule type="colorScale" priority="307">
+    <cfRule type="colorScale" priority="308">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15847,7 +15891,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="308">
+    <cfRule type="colorScale" priority="307">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15859,7 +15903,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q135:R135 H135:O135">
-    <cfRule type="colorScale" priority="311">
+    <cfRule type="colorScale" priority="312">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15869,7 +15913,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="312">
+    <cfRule type="colorScale" priority="311">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15947,6 +15991,16 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q163:R163 H163:N163">
+    <cfRule type="colorScale" priority="329">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="327">
       <colorScale>
         <cfvo type="min"/>
@@ -15967,19 +16021,9 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="329">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q169:R169 H169:N169">
-    <cfRule type="colorScale" priority="333">
+    <cfRule type="colorScale" priority="335">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -15999,51 +16043,7 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="335">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M222">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M226">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="333">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>